<commit_message>
Revert "Merge pull request #79 from Tiger5286/oosaki"
This reverts commit 3680efed7e2e07937ba9b96423766dc390d4b8d2, reversing
changes made to 27f403c073555a480c92f1c6e0f3b8433c0156ae.
</commit_message>
<xml_diff>
--- a/コスト表（改）.xlsx
+++ b/コスト表（改）.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Fall3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AyumuKaminaga\Documents\GitHub\Fall3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0E6020-05AE-4D2C-834A-F8866784AF7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E4B207-16D4-412C-860A-D4418657E519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4C536231-C66C-4A73-9D9A-B6DFFC0D3CF2}"/>
   </bookViews>
@@ -2229,11 +2229,11 @@
       </c>
       <c r="L2" s="53">
         <f>SUMIF(H2:H72,"完了",F2:F72)</f>
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="M2" s="53">
         <f>K2-L2</f>
-        <v>23.099999999999994</v>
+        <v>20.599999999999994</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.4">
@@ -2307,11 +2307,11 @@
       </c>
       <c r="L4" s="53">
         <f>SUMIFS(F2:F72,E2:E72,"アルファ",H2:H72,"完了")</f>
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="53">
         <f t="shared" si="0"/>
-        <v>7.6000000000000014</v>
+        <v>5.1000000000000014</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.4">
@@ -2596,11 +2596,11 @@
       </c>
       <c r="L11" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"上永",H2:H72,"完了")</f>
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="M11" s="80">
         <f t="shared" ref="M11:M14" si="1">K11 - L11</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11" s="79"/>
       <c r="O11" s="95" t="s">
@@ -2652,11 +2652,11 @@
       </c>
       <c r="L12" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"川浪",H2:H72,"完了")</f>
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="M12" s="80">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N12" s="79"/>
       <c r="O12" s="96" t="s">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="L13" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"佐々木",H2:H72,"完了")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M13" s="80">
         <f t="shared" si="1"/>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="N13" s="79"/>
       <c r="O13" s="97" t="s">
@@ -2945,11 +2945,11 @@
       </c>
       <c r="L18" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"上永",E2:E72,"アルファ",H2:H72,"完了")</f>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="M18" s="80">
         <f t="shared" ref="M18:M21" si="3">K18 - L18</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" s="79"/>
       <c r="O18" s="95" t="s">
@@ -2998,11 +2998,11 @@
       </c>
       <c r="L19" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"川浪",E2:E72,"アルファ",H2:H72,"完了")</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M19" s="80">
         <f t="shared" si="3"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="O19" s="96" t="s">
         <v>73</v>
@@ -3052,11 +3052,11 @@
       </c>
       <c r="L20" s="80">
         <f>SUMIFS(F2:F72,A2:A72,"佐々木",E2:E72,"アルファ",H2:H72,"完了")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="80">
         <f>K20 - L20</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="O20" s="97" t="s">
         <v>72</v>
@@ -3785,9 +3785,11 @@
       <c r="F38" s="25">
         <v>0.5</v>
       </c>
-      <c r="G38" s="26"/>
+      <c r="G38" s="26">
+        <v>0.5</v>
+      </c>
       <c r="H38" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="K38" s="74"/>
     </row>
@@ -3808,9 +3810,11 @@
       <c r="F39" s="25">
         <v>0.5</v>
       </c>
-      <c r="G39" s="26"/>
+      <c r="G39" s="26">
+        <v>0.5</v>
+      </c>
       <c r="H39" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="K39" s="74"/>
     </row>
@@ -3994,9 +3998,11 @@
       <c r="F47" s="25">
         <v>0.5</v>
       </c>
-      <c r="G47" s="26"/>
+      <c r="G47" s="26">
+        <v>0.5</v>
+      </c>
       <c r="H47" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.4">
@@ -4016,9 +4022,11 @@
       <c r="F48" s="25">
         <v>0.5</v>
       </c>
-      <c r="G48" s="24"/>
+      <c r="G48" s="24">
+        <v>0.5</v>
+      </c>
       <c r="H48" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.4">
@@ -4284,9 +4292,11 @@
       <c r="F59" s="53">
         <v>0.5</v>
       </c>
-      <c r="G59" s="63"/>
+      <c r="G59" s="63">
+        <v>0.5</v>
+      </c>
       <c r="H59" s="44" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.4">

</xml_diff>